<commit_message>
update stage control and image grabber
</commit_message>
<xml_diff>
--- a/cad/order_list.xlsx
+++ b/cad/order_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a37467f2c57c349/Documenten/fpg/cad/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a37467f2c57c349/Documenten/Python Scripts/wavefrontsensor/cad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{C318CB30-E513-4446-8896-730F00C5D679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{251C246F-E9B1-4E95-94E1-69DDD9C12E91}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{C318CB30-E513-4446-8896-730F00C5D679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B168D5D-1CE6-439D-AC72-B8CFBC86EFDB}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1104" windowWidth="21600" windowHeight="11232" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="82">
   <si>
     <t xml:space="preserve">https://www.bol.com/nl/nl/p/diy-cnc-machine-kit-3018-500mw-grbl-controle-3-as-frees/9300000197781885/?bltgh=pVm1TEkKi3j62aCUsChM9Q.4_8.11.ProductTitle </t>
   </si>
@@ -196,9 +196,6 @@
     <t xml:space="preserve">https://www.tech-specialist.com/nl/type-isb/profielverbinders-isb/rechte-hoekverbinders-isb/hoekverbinders-isb/rechte-hoekverbinders-isb-hoekverbinder-set-sleuf-8-40x40-1007700 </t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.verpas.nl/trillingsdempers/rubber-cilindrisch/type-d/trildemper-type-d-d30-h30-m8x20/?_gl=1*1ouhg48*_up*MQ..*_gs*MQ..&amp;gclid=Cj0KCQjwgIXCBhDBARIsAELC9ZgDzhQ8AI-kzThq1t7ojXjnS-qBSv9FGDjop-RPMeQXwBRQRhbdBxAaAoQwEALw_wcB&amp;gbraid=0AAAAACxAaQuX4otb7hDyn8wndoi7cfDDs </t>
-  </si>
-  <si>
     <t>trillingsdempers</t>
   </si>
   <si>
@@ -281,13 +278,19 @@
   </si>
   <si>
     <t>total to spend</t>
+  </si>
+  <si>
+    <t>https://www.bol.com/nl/nl/p/fsw-products-4-stuks-rubberen-voetjes-onderzetters-rubber-dopje-meubelonderzetter-trillingsdempers-antislip-15-x-12-x-8-mm/9300000102599653/?s2a=&amp;bltgh=piqGyRM2LiqZrGJ8ulxK6Q.4_42_43.44.FeatureOptionButton#productTitle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                     </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -326,13 +329,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="0" tint="-0.34998626667073579"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -348,13 +365,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -813,7 +833,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -890,7 +910,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D9">
         <f>SUM(D2:D8)</f>
@@ -899,7 +919,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -914,7 +934,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -929,7 +949,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -952,7 +972,7 @@
       <c r="C14">
         <v>0.41</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="6">
         <f t="shared" si="1"/>
         <v>10.25</v>
       </c>
@@ -970,7 +990,7 @@
       <c r="C15">
         <v>0.56999999999999995</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="6">
         <f t="shared" si="1"/>
         <v>1.71</v>
       </c>
@@ -980,7 +1000,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B16">
         <v>22</v>
@@ -988,12 +1008,12 @@
       <c r="C16">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="6">
         <f t="shared" si="1"/>
         <v>12.100000000000001</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -1018,7 +1038,7 @@
       <c r="C18">
         <v>71.62</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="6">
         <f t="shared" si="1"/>
         <v>71.62</v>
       </c>
@@ -1028,7 +1048,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B19">
         <v>2</v>
@@ -1036,7 +1056,7 @@
       <c r="C19">
         <v>53.75</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="6">
         <f t="shared" si="1"/>
         <v>107.5</v>
       </c>
@@ -1054,7 +1074,7 @@
       <c r="C20">
         <v>2.4900000000000002</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="6">
         <f t="shared" si="1"/>
         <v>29.880000000000003</v>
       </c>
@@ -1072,7 +1092,7 @@
       <c r="C21">
         <v>4.82</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="6">
         <f t="shared" si="1"/>
         <v>38.56</v>
       </c>
@@ -1082,7 +1102,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B22">
         <v>4</v>
@@ -1090,114 +1110,113 @@
       <c r="C22">
         <v>1.1157999999999999</v>
       </c>
-      <c r="D22">
-        <f t="shared" si="1"/>
-        <v>4.4631999999999996</v>
+      <c r="D22" s="6" t="s">
+        <v>81</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>52</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D23">
         <f>SUM(D11:D22)</f>
-        <v>476.08319999999998</v>
+        <v>471.62</v>
       </c>
       <c r="E23" s="1"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="1"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26">
+      <c r="B26" s="5">
         <v>2</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="5">
         <v>1006</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="5">
         <f t="shared" ref="D26:D28" si="2">B26*C26</f>
         <v>2012</v>
       </c>
-      <c r="E26" s="1"/>
-      <c r="G26" t="s">
+      <c r="E26" s="8"/>
+      <c r="G26" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I26" s="5">
+        <v>1425</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="I26">
-        <v>1425</v>
-      </c>
-      <c r="J26" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27">
+    </row>
+    <row r="27" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="5">
         <v>2</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="5">
         <v>500</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="5">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>62</v>
-      </c>
-      <c r="B28">
+      <c r="E27" s="8"/>
+    </row>
+    <row r="28" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="5">
         <v>0</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="5">
         <v>500</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="E28" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B29">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30">
+      <c r="D30" s="5">
         <f>SUM(D26:D29)</f>
         <v>3012</v>
       </c>
-      <c r="K30" t="s">
-        <v>80</v>
-      </c>
-      <c r="M30">
+      <c r="K30" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="M30" s="5">
         <f>SUM(D30,D23,D9)</f>
-        <v>5282.3732</v>
+        <v>5277.91</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
@@ -1205,12 +1224,12 @@
     </row>
     <row r="32" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="5">
         <v>2</v>
@@ -1223,12 +1242,12 @@
         <v>4492</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="34" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B34" s="5">
         <v>1</v>
@@ -1243,7 +1262,7 @@
     </row>
     <row r="35" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B35" s="5">
         <v>2</v>
@@ -1258,7 +1277,7 @@
     </row>
     <row r="36" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B36" s="5">
         <v>1</v>
@@ -1273,7 +1292,7 @@
     </row>
     <row r="37" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B37" s="5">
         <v>1</v>
@@ -1298,19 +1317,19 @@
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
+    <row r="40" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
+    <row r="41" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>75</v>
+    <row r="42" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
@@ -1357,9 +1376,10 @@
     <hyperlink ref="E18" r:id="rId11" xr:uid="{A03F00E4-E516-4704-A1CF-E6ECBA5C45DB}"/>
     <hyperlink ref="E20" r:id="rId12" xr:uid="{1D9A306D-F0E2-43F1-9885-51AE3DB53FCB}"/>
     <hyperlink ref="E21" r:id="rId13" xr:uid="{6ECC7101-B135-410A-B0CB-AD0B66E8B412}"/>
-    <hyperlink ref="E22" r:id="rId14" display="https://www.verpas.nl/trillingsdempers/rubber-cilindrisch/type-d/trildemper-type-d-d30-h30-m8x20/?_gl=1*1ouhg48*_up*MQ..*_gs*MQ..&amp;gclid=Cj0KCQjwgIXCBhDBARIsAELC9ZgDzhQ8AI-kzThq1t7ojXjnS-qBSv9FGDjop-RPMeQXwBRQRhbdBxAaAoQwEALw_wcB&amp;gbraid=0AAAAACxAaQuX4otb7hDyn8wndoi7cfDDs " xr:uid="{03B3A896-786D-4C6E-A27A-7BECB4150400}"/>
-    <hyperlink ref="E16" r:id="rId15" xr:uid="{88E3CC2F-5D1E-424F-B4A4-35881535C2C4}"/>
-    <hyperlink ref="A42" r:id="rId16" location="productTitle " xr:uid="{6C24FA96-FFAD-4CD0-9980-193712884D0A}"/>
+    <hyperlink ref="E16" r:id="rId14" xr:uid="{88E3CC2F-5D1E-424F-B4A4-35881535C2C4}"/>
+    <hyperlink ref="A42" r:id="rId15" location="productTitle " xr:uid="{6C24FA96-FFAD-4CD0-9980-193712884D0A}"/>
+    <hyperlink ref="A40" r:id="rId16" location="searchTrackingMasterId=Product.100342277&amp;searchTrackingTitle=Cirkelzaagblad+%C3%98210+mm&amp;searchTrackingPageSize=48&amp;searchTrackingPage=1&amp;searchTrackingEvent=click&amp;searchTrackingId=Product.100342277&amp;searchTrackingOrigPos=1&amp;searchTrackingPos=12&amp;searchTrackingOrigPageSize=48&amp;searchTrackingChannel=NL&amp;list=/h/elektrische-zaagmachines/h10070756" display="https://www.lidl.nl/p/parkside-cirkelzaagblad-o210-mm/p100342277#searchTrackingMasterId=Product.100342277&amp;searchTrackingTitle=Cirkelzaagblad+%C3%98210+mm&amp;searchTrackingPageSize=48&amp;searchTrackingPage=1&amp;searchTrackingEvent=click&amp;searchTrackingId=Product.100342277&amp;searchTrackingOrigPos=1&amp;searchTrackingPos=12&amp;searchTrackingOrigPageSize=48&amp;searchTrackingChannel=NL&amp;list=/h/elektrische-zaagmachines/h10070756" xr:uid="{5548155A-4D67-4224-93E7-DCEC293BC4C6}"/>
+    <hyperlink ref="A41" r:id="rId17" display="https://www.hbm-machines.com/nl/p/hbm-professionele-7-delige-boor-tapset?sku=3463&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=19587892072&amp;kb=ga_pm_19587892072_&amp;gad_source=1&amp;gad_campaignid=19580134296&amp;gbraid=0AAAAADvcfwKL1bG_LzTRf5mzlkm2bcHdr&amp;gclid=Cj0KCQjwgIXCBhDBARIsAELC9ZjDkkkRfTDrUvpVQuldNHOdiiOtXC9IySDP-JWY8F3HzUT3H3DzwEAaAhLsEALw_wcB" xr:uid="{775EFE7E-AB5C-4D0F-98D8-8808B138FC78}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>